<commit_message>
Clarify tabletop launch kit and email signup
</commit_message>
<xml_diff>
--- a/public/downloads/launch-kit/Tabletop-Launch-Planner.xlsx
+++ b/public/downloads/launch-kit/Tabletop-Launch-Planner.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start" sheetId="1" r:id="Rc66620e73994437b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding" sheetId="2" r:id="Rfd53224384ff4bc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="3" r:id="R6bf1a59e067c4098"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Costs" sheetId="4" r:id="R309e070144bf4152"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shipping" sheetId="5" r:id="Rd544c11ef9004769"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash" sheetId="6" r:id="R6a18bb9dbf1445ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch plan" sheetId="7" r:id="R95b7acaa216e4558"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ad tests" sheetId="8" r:id="Rf1a5230a0a12471c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R291c2510d9774a13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewers" sheetId="10" r:id="Rdf1aab4771ea4aea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live ops" sheetId="11" r:id="Red89734b8dd546b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="12" r:id="R84a36aa8a96746af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start" sheetId="1" r:id="R2dcb59e409324e2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding" sheetId="2" r:id="R404b0386e1104516"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rewards" sheetId="3" r:id="R23d56680955f4a83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Costs" sheetId="4" r:id="R28107c2559974f33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shipping" sheetId="5" r:id="R219a6bb7d9a042bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash" sheetId="6" r:id="R75662420518e4dc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch plan" sheetId="7" r:id="R1bded3e8ab8448ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ad tests" sheetId="8" r:id="Rca5ba974c3c64436"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="Rd023de4d701b4ec0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewers" sheetId="10" r:id="R7e57e7caa26841bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live ops" sheetId="11" r:id="R7eafdd2c6c664ba8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="12" r:id="R0879d20660a4419e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1150,7 +1150,7 @@
   <x:sheetData>
     <x:row r="1" ht="25" customHeight="1">
       <x:c r="A1" s="7" t="str">
-        <x:v>GUILDFRAME  Tabletop launch planner</x:v>
+        <x:v>GUILDFRAME  Tabletop Campaign Launch Kit</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -1385,7 +1385,7 @@
         <x:v>0.05</x:v>
       </x:c>
       <x:c r="C14" s="8" t="str">
-        <x:v>US default; verify country and current fees</x:v>
+        <x:v>Kickstarter US example; replace for chosen platform</x:v>
       </x:c>
       <x:c r="D14" s="3"/>
       <x:c r="E14" s="3"/>
@@ -1401,7 +1401,7 @@
         <x:v>0.03</x:v>
       </x:c>
       <x:c r="C15" s="8" t="str">
-        <x:v>US standard pledge default</x:v>
+        <x:v>Kickstarter US standard pledge example</x:v>
       </x:c>
       <x:c r="D15" s="3"/>
       <x:c r="E15" s="3"/>
@@ -1514,7 +1514,7 @@
         <x:v>Illustrative combined later collection percentage, verify provider</x:v>
       </x:c>
       <x:c r="D21" s="8" t="str">
-        <x:v>US fees checked 29 Oct 2026: kickstarter.com/help/fees?country=US. All other demo costs are invented planning examples. See Examples and Sources PDF for first party links.</x:v>
+        <x:v>Rates use a Kickstarter US example checked 29 Oct 2026. For Gamefound, replace fees, the small pledge threshold, payout timing and later collection terms. Confirm the actual project setup. See Examples and Sources for both platforms.</x:v>
       </x:c>
       <x:c r="E21" s="8"/>
       <x:c r="F21" s="8"/>
@@ -1611,7 +1611,7 @@
         <x:v>United States</x:v>
       </x:c>
       <x:c r="C27" s="8" t="str">
-        <x:v>Fee defaults below apply only to US campaigns</x:v>
+        <x:v>Fee defaults apply only to Kickstarter US campaigns</x:v>
       </x:c>
       <x:c r="D27" s="8"/>
       <x:c r="E27" s="8"/>
@@ -1729,7 +1729,7 @@
     </x:row>
     <x:row r="37" ht="25" customHeight="1">
       <x:c r="A37" s="8" t="str">
-        <x:v>This model plans one manufactured product SKU used by the physical tiers, plus digital rewards. Cost additional SKUs separately before setting a goal. Demand uses all pledged backers conservatively, while cash deducts expected failed payments. No future sales of remaining inventory are counted as cash.</x:v>
+        <x:v>This model plans one manufactured product SKU used by the physical tiers, plus digital rewards. Cost additional SKUs separately before setting a goal. Demand uses all pledged backers conservatively, while cash deducts expected failed payments. No future sales of remaining inventory are counted as cash. Fees assume one collected transaction per pledge. Installments or multiple charges need an expanded fee and cash schedule.</x:v>
       </x:c>
       <x:c r="B37" s="8"/>
       <x:c r="C37" s="8"/>
@@ -2260,7 +2260,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56c901eea25346c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re668f363c3fd46dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2728,8 +2728,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refefbc6a74f744d1"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d38c8625d434a70"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7b8a7843e1e45ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c74461107934488"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3326,7 +3326,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8be0d11840ba45dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf0737856aa34753"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4192,7 +4192,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re59d42babc934b86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8681b6bc03e04dc2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4751,7 +4751,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad220fc297444461"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R235dc62ef5e94554"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5284,8 +5284,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5207ed4b11d94922"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4185fded14004768"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R720c659c095f4910"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3be8a4458eeb47cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5783,7 +5783,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4febb5fcebea40de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88d7047d8cb3452a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6330,7 +6330,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R807921ee33704e7c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31493c6990144352"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7124,7 +7124,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f6c93bfba0c4c17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd6834079e954e65"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7670,8 +7670,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0e936aa15804c48"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c799681c4e84bbd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8963de9810c84c6d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12a0ce7481f04d34"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7723,7 +7723,7 @@
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
       <x:c r="A3" s="9" t="str">
-        <x:v>Create unique Kickstarter referral tags in Promotions and paste the resulting links. Record own site UTMs separately. Attribution is platform reported, not proof of causal or cross device tracking.</x:v>
+        <x:v>Use Kickstarter generated referral tags for Kickstarter. On Gamefound, use its available campaign reporting and links. Keep own site UTMs separate. Platform attribution does not prove causal or cross device tracking.</x:v>
       </x:c>
       <x:c r="B3" s="9"/>
       <x:c r="C3" s="9"/>
@@ -7816,7 +7816,7 @@
         <x:v>Email launch broadcast</x:v>
       </x:c>
       <x:c r="C8" s="37" t="str">
-        <x:v>Paste Kickstarter generated referral URL</x:v>
+        <x:v>Paste chosen platform campaign tracking URL</x:v>
       </x:c>
       <x:c r="D8" s="37" t="str">
         <x:v>Not live</x:v>
@@ -8095,8 +8095,12 @@
       <x:c r="J22" s="3"/>
     </x:row>
     <x:row r="23" ht="25" customHeight="1">
-      <x:c r="A23" s="3"/>
-      <x:c r="B23" s="3"/>
+      <x:c r="A23" s="3" t="str">
+        <x:v>Gamefound fees</x:v>
+      </x:c>
+      <x:c r="B23" s="3" t="str">
+        <x:v>https://help.gamefound.com/article/284-fees-for-projects-funded-on-gamefound</x:v>
+      </x:c>
       <x:c r="C23" s="3"/>
       <x:c r="D23" s="3"/>
       <x:c r="E23" s="3"/>
@@ -8107,8 +8111,12 @@
       <x:c r="J23" s="3"/>
     </x:row>
     <x:row r="24" ht="25" customHeight="1">
-      <x:c r="A24" s="3"/>
-      <x:c r="B24" s="3"/>
+      <x:c r="A24" s="3" t="str">
+        <x:v>Gamefound stages</x:v>
+      </x:c>
+      <x:c r="B24" s="3" t="str">
+        <x:v>https://help.gamefound.com/article/285-getting-started-with-crowdfunding</x:v>
+      </x:c>
       <x:c r="C24" s="3"/>
       <x:c r="D24" s="3"/>
       <x:c r="E24" s="3"/>
@@ -8119,8 +8127,12 @@
       <x:c r="J24" s="3"/>
     </x:row>
     <x:row r="25" ht="25" customHeight="1">
-      <x:c r="A25" s="3"/>
-      <x:c r="B25" s="3"/>
+      <x:c r="A25" s="3" t="str">
+        <x:v>Gamefound testing</x:v>
+      </x:c>
+      <x:c r="B25" s="3" t="str">
+        <x:v>https://help.gamefound.com/article/366-tester-mode</x:v>
+      </x:c>
       <x:c r="C25" s="3"/>
       <x:c r="D25" s="3"/>
       <x:c r="E25" s="3"/>
@@ -8131,8 +8143,12 @@
       <x:c r="J25" s="3"/>
     </x:row>
     <x:row r="26" ht="25" customHeight="1">
-      <x:c r="A26" s="3"/>
-      <x:c r="B26" s="3"/>
+      <x:c r="A26" s="3" t="str">
+        <x:v>Closing rules</x:v>
+      </x:c>
+      <x:c r="B26" s="3" t="str">
+        <x:v>https://help.gamefound.com/article/434-endgame</x:v>
+      </x:c>
       <x:c r="C26" s="3"/>
       <x:c r="D26" s="3"/>
       <x:c r="E26" s="3"/>
@@ -8141,6 +8157,38 @@
       <x:c r="H26" s="3"/>
       <x:c r="I26" s="3"/>
       <x:c r="J26" s="3"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>Gamefound fees</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>https://help.gamefound.com/article/284-fees-for-projects-funded-on-gamefound</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>Gamefound stages</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>https://help.gamefound.com/article/285-getting-started-with-crowdfunding</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>Gamefound testing</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>https://help.gamefound.com/article/366-tester-mode</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>Closing rules</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>https://help.gamefound.com/article/434-endgame</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -8152,10 +8200,18 @@
     <x:mergeCell ref="B20:F20"/>
     <x:mergeCell ref="B21:F21"/>
     <x:mergeCell ref="B22:F22"/>
+    <x:mergeCell ref="B23:F23"/>
+    <x:mergeCell ref="B24:F24"/>
+    <x:mergeCell ref="B25:F25"/>
+    <x:mergeCell ref="B26:F26"/>
+    <x:mergeCell ref="B27:F27"/>
+    <x:mergeCell ref="B28:F28"/>
+    <x:mergeCell ref="B29:F29"/>
+    <x:mergeCell ref="B30:F30"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf03d10a927dc46d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73de108976be41a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>